<commit_message>
updates for leakage memo
</commit_message>
<xml_diff>
--- a/Extras/2026-05-04 - FLiBe Li7 Study/FLiBe Li7 Results.xlsx
+++ b/Extras/2026-05-04 - FLiBe Li7 Study/FLiBe Li7 Results.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\patri\projects\emma-openmc\Extras\2026-05-04 - FLiBe Li7 Study\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26D298AF-82E4-4EC9-8C1F-80CFA8241349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27DDF933-5E18-405B-9F42-B49263C2B0A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="25">
   <si>
     <t>Blanket</t>
   </si>
@@ -85,6 +96,21 @@
   </si>
   <si>
     <t>Leaked n/src-n</t>
+  </si>
+  <si>
+    <t>Fertile kg/yr</t>
+  </si>
+  <si>
+    <t>U235</t>
+  </si>
+  <si>
+    <t>For 1000 kg/m3</t>
+  </si>
+  <si>
+    <t>(n,fis)/src-n</t>
+  </si>
+  <si>
+    <t>Total (n,fis)/src-n</t>
   </si>
 </sst>
 </file>
@@ -128,9 +154,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -411,17 +438,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A4:O9"/>
+  <dimension ref="A4:T16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" customWidth="1"/>
     <col min="5" max="5" width="2.21875" customWidth="1"/>
-    <col min="8" max="8" width="10.33203125" customWidth="1"/>
-    <col min="10" max="10" width="2.21875" customWidth="1"/>
+    <col min="10" max="10" width="10.33203125" customWidth="1"/>
     <col min="14" max="14" width="2.21875" customWidth="1"/>
+    <col min="18" max="18" width="2.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>5</v>
       </c>
@@ -439,14 +466,20 @@
       <c r="H4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="J4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="O4" t="s">
+      <c r="S4" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -472,17 +505,35 @@
       <c r="I5" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="J5" s="1" t="s">
+        <v>16</v>
+      </c>
       <c r="K5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="O5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="L5" s="1" t="s">
+      <c r="P5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="M5" s="1" t="s">
+      <c r="Q5" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="S5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="T5" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -495,8 +546,48 @@
       <c r="D6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="F6">
+        <v>0.108954927972483</v>
+      </c>
+      <c r="G6" s="2">
+        <v>2.01396393623147E-5</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>1006.8496270316</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <f>O6-P6</f>
+        <v>1006.8496270316</v>
+      </c>
+      <c r="S6">
+        <v>4.2192729999999901E-2</v>
+      </c>
+      <c r="T6" s="2">
+        <v>2.3644361202756801E-5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -509,8 +600,48 @@
       <c r="D7">
         <v>1000</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="F7">
+        <v>8.3009676050873005E-2</v>
+      </c>
+      <c r="G7" s="2">
+        <v>1.7800454467309999E-5</v>
+      </c>
+      <c r="H7">
+        <v>1.1804389805533699</v>
+      </c>
+      <c r="I7">
+        <v>2.3872931118080001E-4</v>
+      </c>
+      <c r="J7">
+        <v>5241.0309329314896</v>
+      </c>
+      <c r="K7">
+        <v>1.05993424912954</v>
+      </c>
+      <c r="L7">
+        <v>0.14788484334959401</v>
+      </c>
+      <c r="M7" s="2">
+        <v>2.5402600980351901E-5</v>
+      </c>
+      <c r="O7">
+        <v>2627.8877302646802</v>
+      </c>
+      <c r="P7">
+        <v>1616.9383178128701</v>
+      </c>
+      <c r="Q7">
+        <f t="shared" ref="Q7:Q9" si="0">O7-P7</f>
+        <v>1010.9494124518101</v>
+      </c>
+      <c r="S7">
+        <v>7.4038749999999999E-3</v>
+      </c>
+      <c r="T7" s="2">
+        <v>2.2721082048215801E-5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -523,8 +654,48 @@
       <c r="D8">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="F8">
+        <v>0.108954927972485</v>
+      </c>
+      <c r="G8" s="2">
+        <v>2.0139639368875499E-5</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>1006.84962703161</v>
+      </c>
+      <c r="P8">
+        <v>0</v>
+      </c>
+      <c r="Q8">
+        <f t="shared" si="0"/>
+        <v>1006.84962703161</v>
+      </c>
+      <c r="S8">
+        <v>4.2192729999999901E-2</v>
+      </c>
+      <c r="T8" s="2">
+        <v>2.3644361202756801E-5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>2</v>
       </c>
@@ -536,6 +707,95 @@
       </c>
       <c r="D9">
         <v>1000</v>
+      </c>
+      <c r="F9">
+        <v>8.0283462156907501E-2</v>
+      </c>
+      <c r="G9" s="2">
+        <v>1.3037482923413301E-5</v>
+      </c>
+      <c r="H9">
+        <v>0.99726513095665403</v>
+      </c>
+      <c r="I9">
+        <v>1.2821841715489999E-4</v>
+      </c>
+      <c r="J9">
+        <v>4316.3924908442004</v>
+      </c>
+      <c r="K9">
+        <v>0.55495875250802695</v>
+      </c>
+      <c r="L9">
+        <v>1.39359927238042E-2</v>
+      </c>
+      <c r="M9" s="2">
+        <v>1.73926813013695E-6</v>
+      </c>
+      <c r="O9">
+        <v>1091.9315772366899</v>
+      </c>
+      <c r="P9">
+        <v>142.510661250851</v>
+      </c>
+      <c r="Q9">
+        <f t="shared" si="0"/>
+        <v>949.42091598583897</v>
+      </c>
+      <c r="S9">
+        <v>2.3705899999998999E-3</v>
+      </c>
+      <c r="T9" s="2">
+        <v>4.9590590505367597E-6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="I11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="I12" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="I13" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="H14" t="s">
+        <v>3</v>
+      </c>
+      <c r="I14">
+        <v>5.1578018695522199E-2</v>
+      </c>
+      <c r="J14" s="2">
+        <v>6.5608716573043603E-6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="H15" t="s">
+        <v>21</v>
+      </c>
+      <c r="I15">
+        <f>0.147884843349594-0.0515780186955222</f>
+        <v>9.630682465407181E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="H16" t="s">
+        <v>12</v>
+      </c>
+      <c r="I16">
+        <v>0.14788484334959401</v>
+      </c>
+      <c r="J16" s="2">
+        <v>2.5402600980351901E-5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>